<commit_message>
VCF 9.1 Regulatory Compliance Library updates.
</commit_message>
<xml_diff>
--- a/regulatory-compliance/cloud-foundation/9.1/bsi-200-1/vcf-91-companion-bsi-200-1.xlsx
+++ b/regulatory-compliance/cloud-foundation/9.1/bsi-200-1/vcf-91-companion-bsi-200-1.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="190" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Version 910-20260612-01</t>
+          <t>Version 910-20260623-01</t>
         </is>
       </c>
     </row>
@@ -536,17 +536,16 @@
     </row>
     <row r="9"/>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Disclaimer</t>
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Additional Resources</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>This kit is intended to provide general guidance for organizations that are considering Broadcom solutions. The information contained in this document is for educational and informational purposes only. This document is not intended to provide advice and is provided "AS IS." Broadcom makes no claims, promises, or guarantees about the accuracy, completeness, or adequacy of the information contained herein. Organizations should engage appropriate legal, business, technical, and audit expertise within their specific organization for review of requirements and effectiveness of implementations.
-This material is provided as is and any express or implied warranties, including, but not limited to, the implied warranties of merchantability and fitness for a particular purpose are disclaimed. In no event shall the copyright holder or contributors be liable for any direct, indirect, incidental, special, exemplary, or consequential damages (including, but not limited to, procurement of substitute goods or services; loss of use, data, or profits; or business interruption) however caused and on any theory of liability, whether in contract, strict liability, or tort (including negligence or otherwise) arising in any way out of the use of this software, even if advised of the possibility of such damage. The provider makes no claims, promises, or guarantees about the accuracy, completeness, or adequacy of this sample. Organizations should engage appropriate legal, business, technical, and audit expertise within their specific organization for review of requirements and effectiveness of implementations. You acknowledge that there may be performance or other considerations, and that these examples may make assumptions which may not be valid in your environment or organization.</t>
+          <t>This is one of a library of companion guides that map VMware Cloud Foundation and its advanced services to security and compliance frameworks. For each framework, the guide is published as a spreadsheet, a CSV data file, a Markdown document, and a PDF, together with a Security Configuration Guide crosswalk that identifies the VCF technical hardening settings relevant to that framework. The companion guide library, the VMware Cloud Foundation Security Configuration Guide, and related security documentation, sample scripts, and Q&amp;A are available at https://brcm.tech/vcf-security.</t>
         </is>
       </c>
     </row>
@@ -554,12 +553,28 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>License</t>
+          <t>Disclaimer</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>This kit is intended to provide general guidance for organizations that are considering Broadcom solutions. The information contained in this document is for educational and informational purposes only. This document is not intended to provide advice and is provided "AS IS." Broadcom makes no claims, promises, or guarantees about the accuracy, completeness, or adequacy of the information contained herein. Organizations should engage appropriate legal, business, technical, and audit expertise within their specific organization for review of requirements and effectiveness of implementations.
+This material is provided as is and any express or implied warranties, including, but not limited to, the implied warranties of merchantability and fitness for a particular purpose are disclaimed. In no event shall the copyright holder or contributors be liable for any direct, indirect, incidental, special, exemplary, or consequential damages (including, but not limited to, procurement of substitute goods or services; loss of use, data, or profits; or business interruption) however caused and on any theory of liability, whether in contract, strict liability, or tort (including negligence or otherwise) arising in any way out of the use of this software, even if advised of the possibility of such damage. The provider makes no claims, promises, or guarantees about the accuracy, completeness, or adequacy of this sample. Organizations should engage appropriate legal, business, technical, and audit expertise within their specific organization for review of requirements and effectiveness of implementations. You acknowledge that there may be performance or other considerations, and that these examples may make assumptions which may not be valid in your environment or organization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>License</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Copyright (c) CA, Inc. All rights reserved.
 You are hereby granted a non-exclusive, worldwide, royalty-free license under CA, Inc.'s copyrights to use, copy, modify, and distribute this software in source code or binary form for use in connection with CA, Inc. products.
@@ -568,16 +583,16 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Third Party Identifiers and Mappings</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>This document includes regulatory compliance and security control identifiers from external sources as a convenience to end users. This does not constitute endorsement, in either direction.
 There is not a one-to-one mapping of product capabilities to third-party controls. A product capability, or set of capabilities, may be applicable to multiple controls. Conversely, a control may be satisfied with the use of multiple capabilities.

</xml_diff>